<commit_message>
Revert "Merge branch 'Develop' into KYO-Map&UI"
This reverts commit a01b80310b1a480574bc54504ea823a53c73539d, reversing
changes made to a6c62bf85ecdf7e24a0a7d14125b1ee7a596c6b7.
</commit_message>
<xml_diff>
--- a/Assets/Data/DataTable/02_Skill_Table_fix.xlsx
+++ b/Assets/Data/DataTable/02_Skill_Table_fix.xlsx
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="154">
   <si>
     <t>방어력 공식</t>
   </si>
@@ -496,6 +496,9 @@
   </si>
   <si>
     <t>SKILL_PASSIVE_DESC_4001</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
   <si>
     <t>SKILL_PASSIVE_NAME_3002</t>
@@ -9463,8 +9466,12 @@
       <c r="O5" s="32">
         <v>0.0</v>
       </c>
-      <c r="P5" s="31"/>
-      <c r="Q5" s="34"/>
+      <c r="P5" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q5" s="34" t="s">
+        <v>113</v>
+      </c>
       <c r="R5" s="34"/>
       <c r="S5" s="32"/>
       <c r="T5" s="34"/>
@@ -9490,10 +9497,10 @@
         <v>1002.0</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G6" s="31">
         <v>0.0</v>
@@ -9522,8 +9529,12 @@
       <c r="O6" s="32">
         <v>0.0</v>
       </c>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="34"/>
+      <c r="P6" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q6" s="34" t="s">
+        <v>113</v>
+      </c>
       <c r="R6" s="34"/>
       <c r="S6" s="31"/>
       <c r="T6" s="34"/>
@@ -9549,10 +9560,10 @@
         <v>1003.0</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G7" s="31">
         <v>0.0</v>
@@ -9581,8 +9592,12 @@
       <c r="O7" s="32">
         <v>0.0</v>
       </c>
-      <c r="P7" s="31"/>
-      <c r="Q7" s="34"/>
+      <c r="P7" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q7" s="34" t="s">
+        <v>113</v>
+      </c>
       <c r="R7" s="34"/>
       <c r="S7" s="31"/>
       <c r="T7" s="34"/>
@@ -9605,13 +9620,13 @@
         <v>1.0</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G8" s="31">
         <v>1.0</v>
@@ -9640,8 +9655,12 @@
       <c r="O8" s="32">
         <v>2.0</v>
       </c>
-      <c r="P8" s="31"/>
-      <c r="Q8" s="34"/>
+      <c r="P8" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q8" s="34" t="s">
+        <v>113</v>
+      </c>
       <c r="R8" s="34"/>
       <c r="S8" s="31"/>
       <c r="T8" s="34"/>
@@ -9664,13 +9683,13 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G9" s="31">
         <v>0.0</v>
@@ -9699,8 +9718,12 @@
       <c r="O9" s="32">
         <v>0.0</v>
       </c>
-      <c r="P9" s="31"/>
-      <c r="Q9" s="34"/>
+      <c r="P9" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q9" s="34" t="s">
+        <v>113</v>
+      </c>
       <c r="R9" s="34"/>
       <c r="S9" s="31"/>
       <c r="T9" s="34"/>
@@ -9723,13 +9746,13 @@
         <v>1.0</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G10" s="31">
         <v>0.0</v>
@@ -9758,8 +9781,12 @@
       <c r="O10" s="32">
         <v>0.0</v>
       </c>
-      <c r="P10" s="31"/>
-      <c r="Q10" s="34"/>
+      <c r="P10" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q10" s="34" t="s">
+        <v>113</v>
+      </c>
       <c r="R10" s="34"/>
       <c r="S10" s="31"/>
       <c r="T10" s="34"/>
@@ -9782,13 +9809,13 @@
         <v>1.0</v>
       </c>
       <c r="D11" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G11" s="31">
         <v>0.0</v>
@@ -9820,7 +9847,9 @@
       <c r="P11" s="31">
         <v>3.0001025E7</v>
       </c>
-      <c r="Q11" s="34"/>
+      <c r="Q11" s="34" t="s">
+        <v>113</v>
+      </c>
       <c r="R11" s="34"/>
       <c r="S11" s="31"/>
       <c r="T11" s="34"/>
@@ -9843,13 +9872,13 @@
         <v>1.0</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E12" s="36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G12" s="31"/>
       <c r="H12" s="31"/>
@@ -9884,13 +9913,13 @@
         <v>1.0</v>
       </c>
       <c r="D13" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E13" s="36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F13" s="36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G13" s="31"/>
       <c r="H13" s="31"/>
@@ -9925,13 +9954,13 @@
         <v>1.0</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E14" s="36" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G14" s="31"/>
       <c r="H14" s="31"/>
@@ -9966,13 +9995,13 @@
         <v>1.0</v>
       </c>
       <c r="D15" s="35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E15" s="36" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F15" s="36" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G15" s="31"/>
       <c r="H15" s="31"/>
@@ -10007,13 +10036,13 @@
         <v>1.0</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E16" s="36" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G16" s="31"/>
       <c r="H16" s="31"/>
@@ -10048,13 +10077,13 @@
         <v>1.0</v>
       </c>
       <c r="D17" s="35" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E17" s="36" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F17" s="36" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G17" s="31"/>
       <c r="H17" s="34"/>
@@ -10080,13 +10109,13 @@
         <v>1.0</v>
       </c>
       <c r="D18" s="35" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E18" s="36" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F18" s="36" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G18" s="31"/>
       <c r="H18" s="34"/>
@@ -10112,13 +10141,13 @@
         <v>1.0</v>
       </c>
       <c r="D19" s="35" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E19" s="36" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F19" s="36" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G19" s="31"/>
       <c r="H19" s="34"/>

</xml_diff>

<commit_message>
Reapply "Merge branch 'Develop' into KYO-Map&UI"
This reverts commit 1afbbf10d443cb089d0cc5dbb51894d843e001f6.
</commit_message>
<xml_diff>
--- a/Assets/Data/DataTable/02_Skill_Table_fix.xlsx
+++ b/Assets/Data/DataTable/02_Skill_Table_fix.xlsx
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="153">
   <si>
     <t>방어력 공식</t>
   </si>
@@ -496,9 +496,6 @@
   </si>
   <si>
     <t>SKILL_PASSIVE_DESC_4001</t>
-  </si>
-  <si>
-    <t>-</t>
   </si>
   <si>
     <t>SKILL_PASSIVE_NAME_3002</t>
@@ -9466,12 +9463,8 @@
       <c r="O5" s="32">
         <v>0.0</v>
       </c>
-      <c r="P5" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q5" s="34" t="s">
-        <v>113</v>
-      </c>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="34"/>
       <c r="R5" s="34"/>
       <c r="S5" s="32"/>
       <c r="T5" s="34"/>
@@ -9497,10 +9490,10 @@
         <v>1002.0</v>
       </c>
       <c r="E6" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="F6" s="31" t="s">
         <v>114</v>
-      </c>
-      <c r="F6" s="31" t="s">
-        <v>115</v>
       </c>
       <c r="G6" s="31">
         <v>0.0</v>
@@ -9529,12 +9522,8 @@
       <c r="O6" s="32">
         <v>0.0</v>
       </c>
-      <c r="P6" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q6" s="34" t="s">
-        <v>113</v>
-      </c>
+      <c r="P6" s="31"/>
+      <c r="Q6" s="34"/>
       <c r="R6" s="34"/>
       <c r="S6" s="31"/>
       <c r="T6" s="34"/>
@@ -9560,10 +9549,10 @@
         <v>1003.0</v>
       </c>
       <c r="E7" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="F7" s="31" t="s">
         <v>116</v>
-      </c>
-      <c r="F7" s="31" t="s">
-        <v>117</v>
       </c>
       <c r="G7" s="31">
         <v>0.0</v>
@@ -9592,12 +9581,8 @@
       <c r="O7" s="32">
         <v>0.0</v>
       </c>
-      <c r="P7" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q7" s="34" t="s">
-        <v>113</v>
-      </c>
+      <c r="P7" s="31"/>
+      <c r="Q7" s="34"/>
       <c r="R7" s="34"/>
       <c r="S7" s="31"/>
       <c r="T7" s="34"/>
@@ -9620,13 +9605,13 @@
         <v>1.0</v>
       </c>
       <c r="D8" s="35" t="s">
+        <v>117</v>
+      </c>
+      <c r="E8" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="E8" s="31" t="s">
+      <c r="F8" s="31" t="s">
         <v>119</v>
-      </c>
-      <c r="F8" s="31" t="s">
-        <v>120</v>
       </c>
       <c r="G8" s="31">
         <v>1.0</v>
@@ -9655,12 +9640,8 @@
       <c r="O8" s="32">
         <v>2.0</v>
       </c>
-      <c r="P8" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q8" s="34" t="s">
-        <v>113</v>
-      </c>
+      <c r="P8" s="31"/>
+      <c r="Q8" s="34"/>
       <c r="R8" s="34"/>
       <c r="S8" s="31"/>
       <c r="T8" s="34"/>
@@ -9683,13 +9664,13 @@
         <v>1.0</v>
       </c>
       <c r="D9" s="35" t="s">
+        <v>120</v>
+      </c>
+      <c r="E9" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="E9" s="31" t="s">
+      <c r="F9" s="31" t="s">
         <v>122</v>
-      </c>
-      <c r="F9" s="31" t="s">
-        <v>123</v>
       </c>
       <c r="G9" s="31">
         <v>0.0</v>
@@ -9718,12 +9699,8 @@
       <c r="O9" s="32">
         <v>0.0</v>
       </c>
-      <c r="P9" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q9" s="34" t="s">
-        <v>113</v>
-      </c>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="34"/>
       <c r="R9" s="34"/>
       <c r="S9" s="31"/>
       <c r="T9" s="34"/>
@@ -9746,13 +9723,13 @@
         <v>1.0</v>
       </c>
       <c r="D10" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="E10" s="31" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="F10" s="31" t="s">
         <v>125</v>
-      </c>
-      <c r="F10" s="31" t="s">
-        <v>126</v>
       </c>
       <c r="G10" s="31">
         <v>0.0</v>
@@ -9781,12 +9758,8 @@
       <c r="O10" s="32">
         <v>0.0</v>
       </c>
-      <c r="P10" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="Q10" s="34" t="s">
-        <v>113</v>
-      </c>
+      <c r="P10" s="31"/>
+      <c r="Q10" s="34"/>
       <c r="R10" s="34"/>
       <c r="S10" s="31"/>
       <c r="T10" s="34"/>
@@ -9809,13 +9782,13 @@
         <v>1.0</v>
       </c>
       <c r="D11" s="35" t="s">
+        <v>126</v>
+      </c>
+      <c r="E11" s="31" t="s">
         <v>127</v>
       </c>
-      <c r="E11" s="31" t="s">
+      <c r="F11" s="31" t="s">
         <v>128</v>
-      </c>
-      <c r="F11" s="31" t="s">
-        <v>129</v>
       </c>
       <c r="G11" s="31">
         <v>0.0</v>
@@ -9847,9 +9820,7 @@
       <c r="P11" s="31">
         <v>3.0001025E7</v>
       </c>
-      <c r="Q11" s="34" t="s">
-        <v>113</v>
-      </c>
+      <c r="Q11" s="34"/>
       <c r="R11" s="34"/>
       <c r="S11" s="31"/>
       <c r="T11" s="34"/>
@@ -9872,13 +9843,13 @@
         <v>1.0</v>
       </c>
       <c r="D12" s="35" t="s">
+        <v>129</v>
+      </c>
+      <c r="E12" s="36" t="s">
         <v>130</v>
       </c>
-      <c r="E12" s="36" t="s">
+      <c r="F12" s="36" t="s">
         <v>131</v>
-      </c>
-      <c r="F12" s="36" t="s">
-        <v>132</v>
       </c>
       <c r="G12" s="31"/>
       <c r="H12" s="31"/>
@@ -9913,13 +9884,13 @@
         <v>1.0</v>
       </c>
       <c r="D13" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="E13" s="36" t="s">
+      <c r="F13" s="36" t="s">
         <v>134</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>135</v>
       </c>
       <c r="G13" s="31"/>
       <c r="H13" s="31"/>
@@ -9954,13 +9925,13 @@
         <v>1.0</v>
       </c>
       <c r="D14" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" s="36" t="s">
         <v>136</v>
       </c>
-      <c r="E14" s="36" t="s">
+      <c r="F14" s="36" t="s">
         <v>137</v>
-      </c>
-      <c r="F14" s="36" t="s">
-        <v>138</v>
       </c>
       <c r="G14" s="31"/>
       <c r="H14" s="31"/>
@@ -9995,13 +9966,13 @@
         <v>1.0</v>
       </c>
       <c r="D15" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="E15" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="E15" s="36" t="s">
+      <c r="F15" s="36" t="s">
         <v>140</v>
-      </c>
-      <c r="F15" s="36" t="s">
-        <v>141</v>
       </c>
       <c r="G15" s="31"/>
       <c r="H15" s="31"/>
@@ -10036,13 +10007,13 @@
         <v>1.0</v>
       </c>
       <c r="D16" s="35" t="s">
+        <v>141</v>
+      </c>
+      <c r="E16" s="36" t="s">
         <v>142</v>
       </c>
-      <c r="E16" s="36" t="s">
+      <c r="F16" s="36" t="s">
         <v>143</v>
-      </c>
-      <c r="F16" s="36" t="s">
-        <v>144</v>
       </c>
       <c r="G16" s="31"/>
       <c r="H16" s="31"/>
@@ -10077,13 +10048,13 @@
         <v>1.0</v>
       </c>
       <c r="D17" s="35" t="s">
+        <v>144</v>
+      </c>
+      <c r="E17" s="36" t="s">
         <v>145</v>
       </c>
-      <c r="E17" s="36" t="s">
+      <c r="F17" s="36" t="s">
         <v>146</v>
-      </c>
-      <c r="F17" s="36" t="s">
-        <v>147</v>
       </c>
       <c r="G17" s="31"/>
       <c r="H17" s="34"/>
@@ -10109,13 +10080,13 @@
         <v>1.0</v>
       </c>
       <c r="D18" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="E18" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="E18" s="36" t="s">
+      <c r="F18" s="36" t="s">
         <v>149</v>
-      </c>
-      <c r="F18" s="36" t="s">
-        <v>150</v>
       </c>
       <c r="G18" s="31"/>
       <c r="H18" s="34"/>
@@ -10141,13 +10112,13 @@
         <v>1.0</v>
       </c>
       <c r="D19" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="E19" s="36" t="s">
         <v>151</v>
       </c>
-      <c r="E19" s="36" t="s">
+      <c r="F19" s="36" t="s">
         <v>152</v>
-      </c>
-      <c r="F19" s="36" t="s">
-        <v>153</v>
       </c>
       <c r="G19" s="31"/>
       <c r="H19" s="34"/>

</xml_diff>